<commit_message>
Re-base cutover plan on physical panel schedule (67 panels / 4467 pts)
Drive build_cutover.py off panels_schedule.json instead of the hardcoded
84-controller / 1160-point functional model. Phases are now grouped by physical
area/floor with real panel names and per-phase panel + point counts that sum to
the full I/O (67 panels, 4467 points): P0 central, P1 rooftop/heat-source plant
(idle), P2 occupied floors on economizer (overnight), P3 basement plant/hydronics
+ DHC intake last. Updated stats, risk checklist count, and README.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/red5-dhcp_controller-cutover-plan.xlsx
+++ b/exports/red5-dhcp_controller-cutover-plan.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +42,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -103,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,6 +124,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -509,7 +515,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Migrate 84 Azbil savic-net FX2 field controllers across 11 panels to new DDC in the April–May shoulder season, using OA economizer free-cooling and local manual operation to keep the hotel conditioned throughout.</t>
+          <t>Migrate the hotel's 67 field panels (904 Delta controllers + modules, 4,467 I/O points) from Azbil savic-net FX2 to new DDC in the April–May shoulder season, using OA economizer free-cooling and local manual operation to keep the hotel conditioned throughout.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -528,24 +534,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Field controllers to replace</t>
+          <t>Physical panels to migrate</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>84</t>
+          <t>67</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Field panels (+ head-end)</t>
+          <t>Delta controllers + modules</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>904</t>
         </is>
       </c>
     </row>
@@ -557,7 +563,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1160</t>
+          <t>4,467</t>
         </is>
       </c>
     </row>
@@ -584,7 +590,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Tokyo shoulder-season OA (~10–22 °C, low enthalpy) lets the airside economizer meet the load with no mechanical cooling, so the towers (LCP-CT) and R-1 chiller are already idle and swap cold. Heating is over, so hot-water hydronics are low-risk. DHC stays live as a warm-spell safety net and is migrated last.</t>
+          <t>Tokyo shoulder-season OA (~10–22 °C, low enthalpy) lets the airside economizer meet the load with no mechanical cooling, so the towers and R-1 chiller are already idle and swap cold. Heating is over, so hot-water hydronics are low-risk. DHC stays live as a warm-spell safety net and its intake is migrated last.</t>
         </is>
       </c>
     </row>
@@ -611,15 +617,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -635,20 +643,30 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Panels (controllers)</t>
+          <t>Areas / panels</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
+          <t>Panels</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Shoulder-season state</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Swap method</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Risk</t>
         </is>
@@ -662,25 +680,31 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>March (hot)</t>
+          <t>March (prep)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>BMS-CENTRAL + network backbone</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
+          <t>System / central — 시스템 제어반</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>n/a — runs in parallel</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Stand up new head-end alongside FX2; prefab panels; bench-test programs; point-verify vs I/O list</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Stand up new head-end alongside FX2; prefab panels; bench-test programs; point-verify vs the 4,467-pt I/O list</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>Prep</t>
         </is>
@@ -699,20 +723,26 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>LCP-CT (8) + R-1 / condenser loop in LCP-3637</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Idle — no mechanical cooling</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
+          <t>Penthouse (PH), Heat source (R-1), Plant / misc — RS-PH2-1, RS-PH1-3, CP-PH1-3, RCP-PH1-3, RCP-PH1-2, RCP-PH1-1, CP-PH-1, RS-PH1-1, CP-R-1, P-1, EVU-6</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>734</v>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Idle — no mechanical cooling; rooftop towers / R-1 / OAU off</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>Power down &amp; swap cold; recommission before any warm spell</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -726,157 +756,91 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>April</t>
+          <t>April–May</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>LCP-1F (3), 2F (4), 3F (4), 4F (7) + air-side of HSL/HSH/3637</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Economizer free-cooling carries load</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>AHU→local, fan hand-on, OA damper ~100%; one AHU at a time; guest floors overnight</t>
-        </is>
+          <t>Floor 31, Floor 21, Floor 10, Floor 4, Floor 3, Floor 2, Floor 1 — RS-31-1, RS-21-1, RS-10-1, RCP-4-1, RCP-4-2, RCP-4-3, RCP-4-4, CP-4-4, RS-4-1, RS-4-2, RCP-3-1, RCP-3-2, RS-3-1, RS-3-2A, RS-3-2B, RCP-2-2, RCP-2-3, RS-2-1, RS-2-2, RS-2-3, RCP-1-1, RCP-1-2, RCP-1-3, RS-1-1, RS-1-2</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>2059</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
+          <t>Economizer free-cooling / DHC carries the occupied floors</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>Guest-floor RS/RCP risers to local; swap overnight, one riser/floor at a time</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
           <t>Moderate</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Apr–May</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>LCP-HSL (17), LCP-HSH (11) — pumps / HX / hydronics</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Heating off; only trickle CHW needed</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>One pump local fixed-speed / manual bypass; duty &amp; standby never both down</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Moderate</t>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Apr–May (last)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Basement B1, Basement B2, Basement B3 — RCP-B1-1, RCP-B1-2, RCP-B1-3, RCP-B1-4, RCP-B1-5, CP-B1-2, CP-B1-3, CP-B1-4, RS-B1-1, RS-B1-2, RS-B1-3, RCP-B2-1, RCP-B2-2, RCP-B2-3, RCP-B2-4, CP-B2-3, CP-B2-4, RS-B2-1, RS-B2-2, RS-B2-3, RS-B2-4B, RS-B2-4A, RS-B2-5, RS-B2-6, RS-B2-7, RCP-B3-1, RCP-B3-2, RCP-B3-3, CP-B3-2, RS-B3-1</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>1649</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Heating off; only trickle CHW; DHC live as safety net</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Pumps / HX / hydronics one at a time on local fixed-speed; duty &amp; standby never both down; DHC-intake panels done last with district coordination (low-occupancy weekend)</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Critical</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>May (last)</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>LCP-DHC (7) — DHC chilled-water + steam intake</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Primary source; economizer covers building</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>DHC valves/pumps to local manual + district coordination; low-occupancy weekend</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>any time</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>LCP-PKG (7) — IT / electrical-room packaged DX</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Runs 24/7 (not seasonal)</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>DX to local thermostat; fast one-at-a-time; spare/portable cooling staged</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>any time</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>LCP-LTG (3) — common-area &amp; facade lighting</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Runs to schedule</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Local switch/override; aviation obstruction light on independent circuit — never dark</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
-      </c>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr"/>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>4467</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -915,102 +879,102 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>AHU / OAU fans</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>COS→手元, fan hand-ON, OA damper fixed ~100% (economizer), DHC coil valve left manually crackable</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Warm spell → be able to open the cooling valve within minutes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>CHW / HW pumps</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>One pump hand-ON at fixed speed; DP/bypass set manually</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>Keep duty OR standby always available; protect domestic-hot-water continuity</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Cooling towers / condenser / R-1</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Leave isolated &amp; de-energised</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>None — off-season; recommission before enabling mechanical cooling</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>DHC intake</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Intake isolation + energy valves and pumps to local manual, fixed position</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>Primary source — coordinate with district operator; do this phase last</t>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Primary source — coordinate with district operator; do these basement panels last</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Packaged units (IT/elec rooms)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>DX on local thermostat, continuous run</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>24/7 critical rooms — stage spare/portable cooling; swap one unit at a time</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Lighting</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Local switching / manual override per circuit</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Aviation obstruction light is regulatory life-safety — independent circuit, always lit</t>
         </is>
@@ -1047,50 +1011,50 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Cutover discipline</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Only one system in manual at any time. Guest-facing zones swapped overnight, back-of-house first. Old controller stays landed on a marshalling strip so you can revert to FX2 within minutes. Freeze all scope changes during the window; spares on site.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Never interrupt</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Life-safety interlocks — smoke control, stair pressurization, exhaust — remain live and coordinated with the fire-alarm system. Aviation obstruction light and IT/electrical-room cooling stay energised.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Verify every point</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>The 1,160-point I/O list is the master checklist. Per controller: point-to-point verify each AI/AO/BI/BO, functional-test, then trend 24–48 h before returning to auto.</t>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>The 4,467-point physical I/O schedule is the master checklist. Per panel: point-to-point verify each DO/DI/BTOT/AI/AO, functional-test, then trend 24–48 h before returning to auto.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Weather safety net</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>DHC stays operational until Phase 4, so a warm spell is covered. The sequence guarantees the building always has either economizer free-cooling or the DHC source available.</t>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>DHC stays operational until the final phase, so a warm spell is covered. The sequence guarantees the building always has either economizer free-cooling or the DHC source available.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reflect 26.07.30 panel schedule (floor + equipment served) across DHCP modules
Adds per-panel floor and served-equipment (AC/EVU/SF/EF/PCU) from the 26.07.30
Excel; regroups areas by authoritative floor. Updates panels-io downloadables
(new build_panels_io.py), commissioning sheets and the floor-based cutover plan.
Totals unchanged: 67 panels / 904 modules / 4,467 used / 5,240 cap.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/red5-dhcp_controller-cutover-plan.xlsx
+++ b/exports/red5-dhcp_controller-cutover-plan.xlsx
@@ -685,7 +685,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>System / central — 시스템 제어반</t>
+          <t>System / central head-end (B2F) — 시스템 제어반</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
@@ -723,14 +723,14 @@
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Penthouse (PH), Heat source (R-1), Plant / misc — RS-PH2-1, RS-PH1-3, CP-PH1-3, RCP-PH1-3, RCP-PH1-2, RCP-PH1-1, CP-PH-1, RS-PH1-1, CP-R-1, P-1, EVU-6</t>
+          <t>Penthouse (PH1/PH2) — rooftop plant, R-1 chiller, OAUs — RS-PH2-1, RS-PH1-3, CP-PH1-3, CP-R-1, RCP-PH1-3, RCP-PH1-2, RCP-PH1-1, CP-PH-1, RS-PH1-1</t>
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>734</v>
+        <v>710</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
@@ -761,14 +761,14 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Floor 31, Floor 21, Floor 10, Floor 4, Floor 3, Floor 2, Floor 1 — RS-31-1, RS-21-1, RS-10-1, RCP-4-1, RCP-4-2, RCP-4-3, RCP-4-4, CP-4-4, RS-4-1, RS-4-2, RCP-3-1, RCP-3-2, RS-3-1, RS-3-2A, RS-3-2B, RCP-2-2, RCP-2-3, RS-2-1, RS-2-2, RS-2-3, RCP-1-1, RCP-1-2, RCP-1-3, RS-1-1, RS-1-2</t>
+          <t>Guest &amp; public floors — 31F, 21F, 10F, 4F–1F (incl. EVU-6) — RS-31-1, RS-21-1, RS-10-1, RCP-4-1, RCP-4-2, RCP-4-3, RCP-4-4, CP-4-4, RS-4-1, RS-4-2, RCP-3-1, RCP-3-2, RS-3-1, RS-3-2A, RS-3-2B, RCP-2-2, RCP-2-3, RS-2-1, RS-2-2, RS-2-3, RCP-1-1, RCP-1-2, RCP-1-3, RS-1-1, RS-1-2, EVU-6</t>
         </is>
       </c>
       <c r="D4" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>2059</v>
+        <v>2083</v>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
@@ -799,11 +799,11 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Basement B1, Basement B2, Basement B3 — RCP-B1-1, RCP-B1-2, RCP-B1-3, RCP-B1-4, RCP-B1-5, CP-B1-2, CP-B1-3, CP-B1-4, RS-B1-1, RS-B1-2, RS-B1-3, RCP-B2-1, RCP-B2-2, RCP-B2-3, RCP-B2-4, CP-B2-3, CP-B2-4, RS-B2-1, RS-B2-2, RS-B2-3, RS-B2-4B, RS-B2-4A, RS-B2-5, RS-B2-6, RS-B2-7, RCP-B3-1, RCP-B3-2, RCP-B3-3, CP-B3-2, RS-B3-1</t>
+          <t>Basements B1–B3 — plant, hydronics, DHC intake, packaged units — RCP-B1-1, RCP-B1-2, RCP-B1-3, RCP-B1-4, RCP-B1-5, CP-B1-2, CP-B1-3, CP-B1-4, RS-B1-1, RS-B1-2, RS-B1-3, RCP-B2-1, RCP-B2-2, RCP-B2-3, RCP-B2-4, CP-B2-3, CP-B2-4, RS-B2-1, RS-B2-2, RS-B2-3, RS-B2-4B, RS-B2-4A, RS-B2-5, RS-B2-6, RS-B2-7, RCP-B3-1, RCP-B3-2, RCP-B3-3, CP-B3-2, RS-B3-1, P-1</t>
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E5" s="8" t="n">
         <v>1649</v>

</xml_diff>